<commit_message>
feat(pharmacy): enhance unit measuring support, catalog imports, and add operations manual
- Add unit column to catalog import/export templates and tracking tables
- Support measuring unit in editable drug rows and inventory manager
- Add comprehensive operations and user manual (manual.md)
</commit_message>
<xml_diff>
--- a/pharmacy-catalog-hamle-template.xlsx
+++ b/pharmacy-catalog-hamle-template.xlsx
@@ -401,15 +401,15 @@
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
     <col min="12" max="12" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -430,25 +430,25 @@
         <v>category</v>
       </c>
       <c r="F1" t="str">
-        <v>hamle-input</v>
+        <v>initialStock</v>
       </c>
       <c r="G1" t="str">
-        <v>initialStock</v>
+        <v>amountInStock</v>
       </c>
       <c r="H1" t="str">
-        <v>amountInStock</v>
+        <v>batchNumber</v>
       </c>
       <c r="I1" t="str">
-        <v>batchNumber</v>
+        <v>expiryDate</v>
       </c>
       <c r="J1" t="str">
-        <v>expiryDate</v>
+        <v>dateAddedToStock</v>
       </c>
       <c r="K1" t="str">
-        <v>dateAddedToStock</v>
+        <v>docNo</v>
       </c>
       <c r="L1" t="str">
-        <v>docNo</v>
+        <v>units</v>
       </c>
     </row>
     <row r="2">
@@ -508,11 +508,11 @@
       <c r="F3" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3">
+      <c r="G3">
         <v>20</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -584,11 +584,11 @@
       <c r="F5" t="str">
         <v/>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5">
+      <c r="G5">
         <v>5</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -698,11 +698,11 @@
       <c r="F8" t="str">
         <v/>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
-      <c r="H8">
+      <c r="G8">
         <v>240</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -812,11 +812,11 @@
       <c r="F11" t="str">
         <v/>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11">
+      <c r="G11">
         <v>60</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -888,11 +888,11 @@
       <c r="F13" t="str">
         <v/>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13">
+      <c r="G13">
         <v>320</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -926,11 +926,11 @@
       <c r="F14" t="str">
         <v/>
       </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
-      <c r="H14">
+      <c r="G14">
         <v>30</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1002,11 +1002,11 @@
       <c r="F16" t="str">
         <v/>
       </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16">
+      <c r="G16">
         <v>100</v>
+      </c>
+      <c r="H16" t="str">
+        <v/>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1040,11 +1040,11 @@
       <c r="F17" t="str">
         <v/>
       </c>
-      <c r="G17" t="str">
-        <v/>
-      </c>
-      <c r="H17">
+      <c r="G17">
         <v>100</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
       </c>
       <c r="I17" t="str">
         <v/>
@@ -1116,11 +1116,11 @@
       <c r="F19" t="str">
         <v/>
       </c>
-      <c r="G19" t="str">
-        <v/>
-      </c>
-      <c r="H19">
+      <c r="G19">
         <v>20</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -1192,11 +1192,11 @@
       <c r="F21" t="str">
         <v/>
       </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-      <c r="H21">
+      <c r="G21">
         <v>60</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -1268,11 +1268,11 @@
       <c r="F23" t="str">
         <v/>
       </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
-      <c r="H23">
+      <c r="G23">
         <v>60</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1344,11 +1344,11 @@
       <c r="F25" t="str">
         <v/>
       </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
-      <c r="H25">
+      <c r="G25">
         <v>200</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
       </c>
       <c r="I25" t="str">
         <v/>
@@ -1382,11 +1382,11 @@
       <c r="F26" t="str">
         <v/>
       </c>
-      <c r="G26" t="str">
-        <v/>
-      </c>
-      <c r="H26">
+      <c r="G26">
         <v>30</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
       </c>
       <c r="I26" t="str">
         <v/>
@@ -1420,11 +1420,11 @@
       <c r="F27" t="str">
         <v/>
       </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-      <c r="H27">
+      <c r="G27">
         <v>10</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
       </c>
       <c r="I27" t="str">
         <v/>
@@ -1496,11 +1496,11 @@
       <c r="F29" t="str">
         <v/>
       </c>
-      <c r="G29" t="str">
-        <v/>
-      </c>
-      <c r="H29">
+      <c r="G29">
         <v>10</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
       </c>
       <c r="I29" t="str">
         <v/>
@@ -1572,11 +1572,11 @@
       <c r="F31" t="str">
         <v/>
       </c>
-      <c r="G31" t="str">
-        <v/>
-      </c>
-      <c r="H31">
+      <c r="G31">
         <v>100</v>
+      </c>
+      <c r="H31" t="str">
+        <v/>
       </c>
       <c r="I31" t="str">
         <v/>
@@ -1610,11 +1610,11 @@
       <c r="F32" t="str">
         <v/>
       </c>
-      <c r="G32" t="str">
-        <v/>
-      </c>
-      <c r="H32">
+      <c r="G32">
         <v>552</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
       </c>
       <c r="I32" t="str">
         <v/>
@@ -1648,11 +1648,11 @@
       <c r="F33" t="str">
         <v/>
       </c>
-      <c r="G33" t="str">
-        <v/>
-      </c>
-      <c r="H33">
+      <c r="G33">
         <v>90</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -1876,11 +1876,11 @@
       <c r="F39" t="str">
         <v/>
       </c>
-      <c r="G39" t="str">
-        <v/>
-      </c>
-      <c r="H39">
+      <c r="G39">
         <v>100</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
       </c>
       <c r="I39" t="str">
         <v/>
@@ -1914,11 +1914,11 @@
       <c r="F40" t="str">
         <v/>
       </c>
-      <c r="G40" t="str">
-        <v/>
-      </c>
-      <c r="H40">
+      <c r="G40">
         <v>50</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
       </c>
       <c r="I40" t="str">
         <v/>
@@ -1990,11 +1990,11 @@
       <c r="F42" t="str">
         <v/>
       </c>
-      <c r="G42" t="str">
-        <v/>
-      </c>
-      <c r="H42">
+      <c r="G42">
         <v>100</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
       </c>
       <c r="I42" t="str">
         <v/>
@@ -2028,11 +2028,11 @@
       <c r="F43" t="str">
         <v/>
       </c>
-      <c r="G43" t="str">
-        <v/>
-      </c>
-      <c r="H43">
+      <c r="G43">
         <v>100</v>
+      </c>
+      <c r="H43" t="str">
+        <v/>
       </c>
       <c r="I43" t="str">
         <v/>
@@ -2066,11 +2066,11 @@
       <c r="F44" t="str">
         <v/>
       </c>
-      <c r="G44" t="str">
-        <v/>
-      </c>
-      <c r="H44">
+      <c r="G44">
         <v>5</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -2256,11 +2256,11 @@
       <c r="F49" t="str">
         <v/>
       </c>
-      <c r="G49" t="str">
-        <v/>
-      </c>
-      <c r="H49">
+      <c r="G49">
         <v>100</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
       </c>
       <c r="I49" t="str">
         <v/>
@@ -2294,11 +2294,11 @@
       <c r="F50" t="str">
         <v/>
       </c>
-      <c r="G50" t="str">
-        <v/>
-      </c>
-      <c r="H50">
+      <c r="G50">
         <v>200</v>
+      </c>
+      <c r="H50" t="str">
+        <v/>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -2484,11 +2484,11 @@
       <c r="F55" t="str">
         <v/>
       </c>
-      <c r="G55" t="str">
-        <v/>
-      </c>
-      <c r="H55">
+      <c r="G55">
         <v>20</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
       </c>
       <c r="I55" t="str">
         <v/>
@@ -2598,11 +2598,11 @@
       <c r="F58" t="str">
         <v/>
       </c>
-      <c r="G58" t="str">
-        <v/>
-      </c>
-      <c r="H58">
+      <c r="G58">
         <v>54</v>
+      </c>
+      <c r="H58" t="str">
+        <v/>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2712,11 +2712,11 @@
       <c r="F61" t="str">
         <v/>
       </c>
-      <c r="G61" t="str">
-        <v/>
-      </c>
-      <c r="H61">
+      <c r="G61">
         <v>15</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -2826,11 +2826,11 @@
       <c r="F64" t="str">
         <v/>
       </c>
-      <c r="G64" t="str">
-        <v/>
-      </c>
-      <c r="H64">
+      <c r="G64">
         <v>50</v>
+      </c>
+      <c r="H64" t="str">
+        <v/>
       </c>
       <c r="I64" t="str">
         <v/>
@@ -3092,11 +3092,11 @@
       <c r="F71" t="str">
         <v/>
       </c>
-      <c r="G71" t="str">
-        <v/>
-      </c>
-      <c r="H71">
+      <c r="G71">
         <v>100</v>
+      </c>
+      <c r="H71" t="str">
+        <v/>
       </c>
       <c r="I71" t="str">
         <v/>
@@ -3282,11 +3282,11 @@
       <c r="F76" t="str">
         <v/>
       </c>
-      <c r="G76" t="str">
-        <v/>
-      </c>
-      <c r="H76">
+      <c r="G76">
         <v>30</v>
+      </c>
+      <c r="H76" t="str">
+        <v/>
       </c>
       <c r="I76" t="str">
         <v/>
@@ -3434,11 +3434,11 @@
       <c r="F80" t="str">
         <v/>
       </c>
-      <c r="G80" t="str">
-        <v/>
-      </c>
-      <c r="H80">
+      <c r="G80">
         <v>20</v>
+      </c>
+      <c r="H80" t="str">
+        <v/>
       </c>
       <c r="I80" t="str">
         <v/>
@@ -3472,11 +3472,11 @@
       <c r="F81" t="str">
         <v/>
       </c>
-      <c r="G81" t="str">
-        <v/>
-      </c>
-      <c r="H81">
+      <c r="G81">
         <v>20</v>
+      </c>
+      <c r="H81" t="str">
+        <v/>
       </c>
       <c r="I81" t="str">
         <v/>
@@ -3510,11 +3510,11 @@
       <c r="F82" t="str">
         <v/>
       </c>
-      <c r="G82" t="str">
-        <v/>
-      </c>
-      <c r="H82">
+      <c r="G82">
         <v>100</v>
+      </c>
+      <c r="H82" t="str">
+        <v/>
       </c>
       <c r="I82" t="str">
         <v/>
@@ -3548,11 +3548,11 @@
       <c r="F83" t="str">
         <v/>
       </c>
-      <c r="G83" t="str">
-        <v/>
-      </c>
-      <c r="H83">
+      <c r="G83">
         <v>50</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
       </c>
       <c r="I83" t="str">
         <v/>
@@ -3624,11 +3624,11 @@
       <c r="F85" t="str">
         <v/>
       </c>
-      <c r="G85" t="str">
-        <v/>
-      </c>
-      <c r="H85">
+      <c r="G85">
         <v>10</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
       </c>
       <c r="I85" t="str">
         <v/>
@@ -3966,11 +3966,11 @@
       <c r="F94" t="str">
         <v/>
       </c>
-      <c r="G94" t="str">
-        <v/>
-      </c>
-      <c r="H94">
+      <c r="G94">
         <v>100</v>
+      </c>
+      <c r="H94" t="str">
+        <v/>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -4232,11 +4232,11 @@
       <c r="F101" t="str">
         <v/>
       </c>
-      <c r="G101" t="str">
-        <v/>
-      </c>
-      <c r="H101">
+      <c r="G101">
         <v>2</v>
+      </c>
+      <c r="H101" t="str">
+        <v/>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -4346,11 +4346,11 @@
       <c r="F104" t="str">
         <v/>
       </c>
-      <c r="G104" t="str">
-        <v/>
-      </c>
-      <c r="H104">
+      <c r="G104">
         <v>200</v>
+      </c>
+      <c r="H104" t="str">
+        <v/>
       </c>
       <c r="I104" t="str">
         <v/>
@@ -4460,11 +4460,11 @@
       <c r="F107" t="str">
         <v/>
       </c>
-      <c r="G107" t="str">
-        <v/>
-      </c>
-      <c r="H107">
+      <c r="G107">
         <v>50</v>
+      </c>
+      <c r="H107" t="str">
+        <v/>
       </c>
       <c r="I107" t="str">
         <v/>
@@ -4536,11 +4536,11 @@
       <c r="F109" t="str">
         <v/>
       </c>
-      <c r="G109" t="str">
-        <v/>
-      </c>
-      <c r="H109">
+      <c r="G109">
         <v>20</v>
+      </c>
+      <c r="H109" t="str">
+        <v/>
       </c>
       <c r="I109" t="str">
         <v/>
@@ -4688,11 +4688,11 @@
       <c r="F113" t="str">
         <v/>
       </c>
-      <c r="G113" t="str">
-        <v/>
-      </c>
-      <c r="H113">
+      <c r="G113">
         <v>33</v>
+      </c>
+      <c r="H113" t="str">
+        <v/>
       </c>
       <c r="I113" t="str">
         <v/>
@@ -4916,11 +4916,11 @@
       <c r="F119" t="str">
         <v/>
       </c>
-      <c r="G119" t="str">
-        <v/>
-      </c>
-      <c r="H119">
+      <c r="G119">
         <v>10</v>
+      </c>
+      <c r="H119" t="str">
+        <v/>
       </c>
       <c r="I119" t="str">
         <v/>
@@ -5068,11 +5068,11 @@
       <c r="F123" t="str">
         <v/>
       </c>
-      <c r="G123" t="str">
-        <v/>
-      </c>
-      <c r="H123">
+      <c r="G123">
         <v>10</v>
+      </c>
+      <c r="H123" t="str">
+        <v/>
       </c>
       <c r="I123" t="str">
         <v/>
@@ -5106,11 +5106,11 @@
       <c r="F124" t="str">
         <v/>
       </c>
-      <c r="G124" t="str">
-        <v/>
-      </c>
-      <c r="H124">
+      <c r="G124">
         <v>10</v>
+      </c>
+      <c r="H124" t="str">
+        <v/>
       </c>
       <c r="I124" t="str">
         <v/>
@@ -5296,11 +5296,11 @@
       <c r="F129" t="str">
         <v/>
       </c>
-      <c r="G129" t="str">
-        <v/>
-      </c>
-      <c r="H129">
+      <c r="G129">
         <v>2</v>
+      </c>
+      <c r="H129" t="str">
+        <v/>
       </c>
       <c r="I129" t="str">
         <v/>
@@ -5410,11 +5410,11 @@
       <c r="F132" t="str">
         <v/>
       </c>
-      <c r="G132" t="str">
-        <v/>
-      </c>
-      <c r="H132">
+      <c r="G132">
         <v>10</v>
+      </c>
+      <c r="H132" t="str">
+        <v/>
       </c>
       <c r="I132" t="str">
         <v/>
@@ -5714,11 +5714,11 @@
       <c r="F140" t="str">
         <v/>
       </c>
-      <c r="G140" t="str">
-        <v/>
-      </c>
-      <c r="H140">
+      <c r="G140">
         <v>30</v>
+      </c>
+      <c r="H140" t="str">
+        <v/>
       </c>
       <c r="I140" t="str">
         <v/>
@@ -5752,11 +5752,11 @@
       <c r="F141" t="str">
         <v/>
       </c>
-      <c r="G141" t="str">
-        <v/>
-      </c>
-      <c r="H141">
+      <c r="G141">
         <v>300</v>
+      </c>
+      <c r="H141" t="str">
+        <v/>
       </c>
       <c r="I141" t="str">
         <v/>
@@ -6018,11 +6018,11 @@
       <c r="F148" t="str">
         <v/>
       </c>
-      <c r="G148" t="str">
-        <v/>
-      </c>
-      <c r="H148">
+      <c r="G148">
         <v>70</v>
+      </c>
+      <c r="H148" t="str">
+        <v/>
       </c>
       <c r="I148" t="str">
         <v/>
@@ -6056,11 +6056,11 @@
       <c r="F149" t="str">
         <v/>
       </c>
-      <c r="G149" t="str">
-        <v/>
-      </c>
-      <c r="H149">
+      <c r="G149">
         <v>50</v>
+      </c>
+      <c r="H149" t="str">
+        <v/>
       </c>
       <c r="I149" t="str">
         <v/>

</xml_diff>